<commit_message>
feat: add brand block
</commit_message>
<xml_diff>
--- a/parsing/data/brands-import.xlsx
+++ b/parsing/data/brands-import.xlsx
@@ -436,7 +436,7 @@
         <v>drl</v>
       </c>
       <c r="C2" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/09/mAAAAgDI6OA-960.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-incandescent_light_bulb.svg.png</v>
       </c>
       <c r="D2" t="str">
         <v>ремонт фар дхо</v>
@@ -465,7 +465,7 @@
         <v>acura</v>
       </c>
       <c r="C3" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/acura.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-acura_logo.svg.png</v>
       </c>
       <c r="D3" t="str">
         <v>ремонт фар acura</v>
@@ -494,7 +494,7 @@
         <v>audi</v>
       </c>
       <c r="C4" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/audi.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-audi-logo_2016.svg.png</v>
       </c>
       <c r="D4" t="str">
         <v>ремонт фар audi</v>
@@ -523,7 +523,7 @@
         <v>bentley</v>
       </c>
       <c r="C5" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/bentley.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/bentley-logo.png</v>
       </c>
       <c r="D5" t="str">
         <v>ремонт фар bentley</v>
@@ -552,7 +552,7 @@
         <v>bmw</v>
       </c>
       <c r="C6" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/bmw-100x100.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-bmw.svg.png</v>
       </c>
       <c r="D6" t="str">
         <v>ремонт фар bmw</v>
@@ -581,7 +581,7 @@
         <v>cadillac</v>
       </c>
       <c r="C7" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/cadillac-100x100.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/cadillac-logo.png</v>
       </c>
       <c r="D7" t="str">
         <v>ремонт фар cadillac</v>
@@ -610,7 +610,7 @@
         <v>chevrolet</v>
       </c>
       <c r="C8" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/chevrolet.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-chevrolet-logo.png</v>
       </c>
       <c r="D8" t="str">
         <v>ремонт фар chevrolet</v>
@@ -639,7 +639,7 @@
         <v>chrysler</v>
       </c>
       <c r="C9" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/chrysler.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-chryply_blue_pentastar.svg.png</v>
       </c>
       <c r="D9" t="str">
         <v>ремонт фар chrysler</v>
@@ -668,7 +668,7 @@
         <v>dodge</v>
       </c>
       <c r="C10" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/dodge-100x100.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-dodge_logo.svg.png</v>
       </c>
       <c r="D10" t="str">
         <v>ремонт фар dodge</v>
@@ -697,7 +697,7 @@
         <v>ferrari</v>
       </c>
       <c r="C11" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/ferrari.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ferrari-logo.png</v>
       </c>
       <c r="D11" t="str">
         <v>ремонт фар ferrari</v>
@@ -726,7 +726,7 @@
         <v>ford</v>
       </c>
       <c r="C12" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/ford.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-ford_motor_company_logo.svg.png</v>
       </c>
       <c r="D12" t="str">
         <v>ремонт фар ford</v>
@@ -755,7 +755,7 @@
         <v>honda</v>
       </c>
       <c r="C13" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/honda.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-honda.svg.png</v>
       </c>
       <c r="D13" t="str">
         <v>ремонт фар honda</v>
@@ -784,7 +784,7 @@
         <v>hpl</v>
       </c>
       <c r="C14" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/07/kyaaagkceoa-960.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-incandescent_light_bulb.svg.png</v>
       </c>
       <c r="D14" t="str">
         <v>ремонт фар hpl</v>
@@ -813,7 +813,7 @@
         <v>hummer</v>
       </c>
       <c r="C15" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/hummer.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-hummer.svg.png</v>
       </c>
       <c r="D15" t="str">
         <v>ремонт фар hummer</v>
@@ -842,7 +842,7 @@
         <v>hyundai</v>
       </c>
       <c r="C16" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/hyundai.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-hyundai_motor_company_logo.svg.png</v>
       </c>
       <c r="D16" t="str">
         <v>ремонт фар hyundai</v>
@@ -871,7 +871,7 @@
         <v>infiniti</v>
       </c>
       <c r="C17" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/infiniti.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/infiniti-logo.png</v>
       </c>
       <c r="D17" t="str">
         <v>ремонт фар infiniti</v>
@@ -900,7 +900,7 @@
         <v>jaguar</v>
       </c>
       <c r="C18" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/jaguar.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/jaguar-logo.png</v>
       </c>
       <c r="D18" t="str">
         <v>ремонт фар jaguar</v>
@@ -929,7 +929,7 @@
         <v>jeep</v>
       </c>
       <c r="C19" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/jeep.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-jeep_logo.svg.png</v>
       </c>
       <c r="D19" t="str">
         <v>ремонт фар jeep</v>
@@ -958,7 +958,7 @@
         <v>kia</v>
       </c>
       <c r="C20" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/kia-100x100.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-kia_logo3.svg.png</v>
       </c>
       <c r="D20" t="str">
         <v>ремонт фар kia</v>
@@ -987,7 +987,7 @@
         <v>ktm</v>
       </c>
       <c r="C21" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/ktm.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-ktm-logo.svg.png</v>
       </c>
       <c r="D21" t="str">
         <v>ремонт фар ktm</v>
@@ -1016,7 +1016,7 @@
         <v>land-rover</v>
       </c>
       <c r="C22" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/landrover.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/land-rover-logo.png</v>
       </c>
       <c r="D22" t="str">
         <v>ремонт фар land rover</v>
@@ -1045,7 +1045,7 @@
         <v>lexus</v>
       </c>
       <c r="C23" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/lexus.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/lexus-logo.png</v>
       </c>
       <c r="D23" t="str">
         <v>ремонт фар lexus</v>
@@ -1074,7 +1074,7 @@
         <v>maserati</v>
       </c>
       <c r="C24" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/maseratti.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/maserati-logo.png</v>
       </c>
       <c r="D24" t="str">
         <v>ремонт фар maserati</v>
@@ -1103,7 +1103,7 @@
         <v>maybach</v>
       </c>
       <c r="C25" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/maybach.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-maybach-logo.svg.png</v>
       </c>
       <c r="D25" t="str">
         <v>ремонт фар maybach</v>
@@ -1132,7 +1132,7 @@
         <v>mazda</v>
       </c>
       <c r="C26" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/mazda-100x100.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mazda-logo.png</v>
       </c>
       <c r="D26" t="str">
         <v>ремонт фар mazda</v>
@@ -1161,7 +1161,7 @@
         <v>mercedes</v>
       </c>
       <c r="C27" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/mb.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mercedes-benz-logo.png</v>
       </c>
       <c r="D27" t="str">
         <v>ремонт фар mercedes</v>
@@ -1190,7 +1190,7 @@
         <v>mini</v>
       </c>
       <c r="C28" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-27.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mini-logo.png</v>
       </c>
       <c r="D28" t="str">
         <v>ремонт фар mini</v>
@@ -1219,7 +1219,7 @@
         <v>mitsubishi</v>
       </c>
       <c r="C29" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/mitsubishi.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-mitsubishi_logo.svg.png</v>
       </c>
       <c r="D29" t="str">
         <v>ремонт фар mitsubishi</v>
@@ -1248,7 +1248,7 @@
         <v>nissan</v>
       </c>
       <c r="C30" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/nissan-100x100.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-nissan_logo.svg.png</v>
       </c>
       <c r="D30" t="str">
         <v>ремонт фар nissan</v>
@@ -1277,7 +1277,7 @@
         <v>opel</v>
       </c>
       <c r="C31" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/opel-100x100.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-opel_logo_2023.svg.png</v>
       </c>
       <c r="D31" t="str">
         <v>ремонт фар opel</v>
@@ -1306,7 +1306,7 @@
         <v>peugeot</v>
       </c>
       <c r="C32" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/peugeot.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/peugeot-logo.png</v>
       </c>
       <c r="D32" t="str">
         <v>ремонт фар peugeot</v>
@@ -1335,7 +1335,7 @@
         <v>porsche</v>
       </c>
       <c r="C33" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/porsche.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/porsche-logo.png</v>
       </c>
       <c r="D33" t="str">
         <v>ремонт фар porsche</v>
@@ -1364,7 +1364,7 @@
         <v>renault</v>
       </c>
       <c r="C34" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2021/10/renault-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/renault-logo.png</v>
       </c>
       <c r="D34" t="str">
         <v>ремонт фар renault</v>
@@ -1393,7 +1393,7 @@
         <v>rolls-royce</v>
       </c>
       <c r="C35" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/rolls-r.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-rolls-royce_motor_cars_logo.svg.png</v>
       </c>
       <c r="D35" t="str">
         <v>ремонт фар rolls-royce</v>
@@ -1422,7 +1422,7 @@
         <v>saab</v>
       </c>
       <c r="C36" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/N-AAAgKn-A-9601.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/saab-logo.png</v>
       </c>
       <c r="D36" t="str">
         <v>ремонт фар saab</v>
@@ -1451,7 +1451,7 @@
         <v>skoda</v>
       </c>
       <c r="C37" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/skoda-100x100.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/skoda-logo.png</v>
       </c>
       <c r="D37" t="str">
         <v>ремонт фар skoda</v>
@@ -1480,7 +1480,7 @@
         <v>ssangyong</v>
       </c>
       <c r="C38" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2023/03/EmP6Qa8cqkZIT6R_qVvDnhI6ps8-960.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ssangyong-logo.png</v>
       </c>
       <c r="D38" t="str">
         <v>ремонт фар ssangyong</v>
@@ -1509,7 +1509,7 @@
         <v>subaru</v>
       </c>
       <c r="C39" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/subaru.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/subaru-logo.png</v>
       </c>
       <c r="D39" t="str">
         <v>ремонт фар subaru</v>
@@ -1538,7 +1538,7 @@
         <v>suzuki</v>
       </c>
       <c r="C40" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/suzuki.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/suzuki-logo.png</v>
       </c>
       <c r="D40" t="str">
         <v>ремонт фар suzuki</v>
@@ -1567,7 +1567,7 @@
         <v>toyota</v>
       </c>
       <c r="C41" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/toyota.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-toyota.svg.png</v>
       </c>
       <c r="D41" t="str">
         <v>ремонт фар toyota</v>
@@ -1596,7 +1596,7 @@
         <v>vw</v>
       </c>
       <c r="C42" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/vw.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-volkswagen_logo_2019.svg.png</v>
       </c>
       <c r="D42" t="str">
         <v>ремонт фар volkswagen</v>
@@ -1625,7 +1625,7 @@
         <v>volvo</v>
       </c>
       <c r="C43" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/volvo.jpg</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-volvo_logo.svg.png</v>
       </c>
       <c r="D43" t="str">
         <v>ремонт фар volvo</v>

</xml_diff>

<commit_message>
fix: brands block homepage
</commit_message>
<xml_diff>
--- a/parsing/data/brands-import.xlsx
+++ b/parsing/data/brands-import.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,1225 +430,1167 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ДХО</v>
+        <v>ACURA</v>
       </c>
       <c r="B2" t="str">
-        <v>drl</v>
+        <v>acura</v>
       </c>
       <c r="C2" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-incandescent_light_bulb.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/acura.svg</v>
       </c>
       <c r="D2" t="str">
-        <v>ремонт фар дхо</v>
+        <v>ремонт фар acura</v>
       </c>
       <c r="E2" t="str">
-        <v>Ремонт и тюнинг фар ДХО в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
       </c>
       <c r="F2" t="str">
-        <v>Ремонт и тюнинг фар ДХО в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар ACURA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G2" t="str">
-        <v>ремонт фар дхо, ремонт фар дхо спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар acura, ремонт фар acura спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H2" t="str">
-        <v>Ремонт и тюнинг фар ДХО в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
       </c>
       <c r="I2" t="str">
-        <v>Ремонт и тюнинг фар ДХО в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ACURA</v>
+        <v>AUDI</v>
       </c>
       <c r="B3" t="str">
-        <v>acura</v>
+        <v>audi</v>
       </c>
       <c r="C3" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-acura_logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/audi-logo.svg</v>
       </c>
       <c r="D3" t="str">
-        <v>ремонт фар acura</v>
+        <v>ремонт фар audi</v>
       </c>
       <c r="E3" t="str">
-        <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
       </c>
       <c r="F3" t="str">
-        <v>Ремонт и тюнинг фар ACURA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар AUDI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G3" t="str">
-        <v>ремонт фар acura, ремонт фар acura спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар audi, ремонт фар audi спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H3" t="str">
-        <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
       </c>
       <c r="I3" t="str">
-        <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>AUDI</v>
+        <v>BENTLEY</v>
       </c>
       <c r="B4" t="str">
-        <v>audi</v>
+        <v>bentley</v>
       </c>
       <c r="C4" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-audi-logo_2016.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/bentley_logo.svg</v>
       </c>
       <c r="D4" t="str">
-        <v>ремонт фар audi</v>
+        <v>ремонт фар bentley</v>
       </c>
       <c r="E4" t="str">
-        <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
       </c>
       <c r="F4" t="str">
-        <v>Ремонт и тюнинг фар AUDI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар BENTLEY в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G4" t="str">
-        <v>ремонт фар audi, ремонт фар audi спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар bentley, ремонт фар bentley спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H4" t="str">
-        <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
       </c>
       <c r="I4" t="str">
-        <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BENTLEY</v>
+        <v>BMW</v>
       </c>
       <c r="B5" t="str">
-        <v>bentley</v>
+        <v>bmw</v>
       </c>
       <c r="C5" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/bentley-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/bmw.svg</v>
       </c>
       <c r="D5" t="str">
-        <v>ремонт фар bentley</v>
+        <v>ремонт фар bmw</v>
       </c>
       <c r="E5" t="str">
-        <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
       </c>
       <c r="F5" t="str">
-        <v>Ремонт и тюнинг фар BENTLEY в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар BMW в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G5" t="str">
-        <v>ремонт фар bentley, ремонт фар bentley спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар bmw, ремонт фар bmw спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H5" t="str">
-        <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
       </c>
       <c r="I5" t="str">
-        <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BMW</v>
+        <v>CADILLAC</v>
       </c>
       <c r="B6" t="str">
-        <v>bmw</v>
+        <v>cadillac</v>
       </c>
       <c r="C6" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-bmw.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/cadillac.svg</v>
       </c>
       <c r="D6" t="str">
-        <v>ремонт фар bmw</v>
+        <v>ремонт фар cadillac</v>
       </c>
       <c r="E6" t="str">
-        <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
       </c>
       <c r="F6" t="str">
-        <v>Ремонт и тюнинг фар BMW в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар CADILLAC в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G6" t="str">
-        <v>ремонт фар bmw, ремонт фар bmw спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар cadillac, ремонт фар cadillac спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H6" t="str">
-        <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
       </c>
       <c r="I6" t="str">
-        <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>CADILLAC</v>
+        <v>CHEVROLET</v>
       </c>
       <c r="B7" t="str">
-        <v>cadillac</v>
+        <v>chevrolet</v>
       </c>
       <c r="C7" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/cadillac-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/chevrolet.webp</v>
       </c>
       <c r="D7" t="str">
-        <v>ремонт фар cadillac</v>
+        <v>ремонт фар chevrolet</v>
       </c>
       <c r="E7" t="str">
-        <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
       </c>
       <c r="F7" t="str">
-        <v>Ремонт и тюнинг фар CADILLAC в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар CHEVROLET в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G7" t="str">
-        <v>ремонт фар cadillac, ремонт фар cadillac спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар chevrolet, ремонт фар chevrolet спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H7" t="str">
-        <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
       </c>
       <c r="I7" t="str">
-        <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CHEVROLET</v>
+        <v>CHRYSLER</v>
       </c>
       <c r="B8" t="str">
-        <v>chevrolet</v>
+        <v>chrysler</v>
       </c>
       <c r="C8" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-chevrolet-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-chryply_blue_pentastar.svg.png</v>
       </c>
       <c r="D8" t="str">
-        <v>ремонт фар chevrolet</v>
+        <v>ремонт фар chrysler</v>
       </c>
       <c r="E8" t="str">
-        <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
       </c>
       <c r="F8" t="str">
-        <v>Ремонт и тюнинг фар CHEVROLET в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар CHRYSLER в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G8" t="str">
-        <v>ремонт фар chevrolet, ремонт фар chevrolet спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар chrysler, ремонт фар chrysler спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H8" t="str">
-        <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
       </c>
       <c r="I8" t="str">
-        <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>CHRYSLER</v>
+        <v>DODGE</v>
       </c>
       <c r="B9" t="str">
-        <v>chrysler</v>
+        <v>dodge</v>
       </c>
       <c r="C9" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-chryply_blue_pentastar.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/dodge.svg</v>
       </c>
       <c r="D9" t="str">
-        <v>ремонт фар chrysler</v>
+        <v>ремонт фар dodge</v>
       </c>
       <c r="E9" t="str">
-        <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
       </c>
       <c r="F9" t="str">
-        <v>Ремонт и тюнинг фар CHRYSLER в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар DODGE в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G9" t="str">
-        <v>ремонт фар chrysler, ремонт фар chrysler спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар dodge, ремонт фар dodge спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H9" t="str">
-        <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
       </c>
       <c r="I9" t="str">
-        <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>DODGE</v>
+        <v>FERRARI</v>
       </c>
       <c r="B10" t="str">
-        <v>dodge</v>
+        <v>ferrari</v>
       </c>
       <c r="C10" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-dodge_logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ferrari-logo.png</v>
       </c>
       <c r="D10" t="str">
-        <v>ремонт фар dodge</v>
+        <v>ремонт фар ferrari</v>
       </c>
       <c r="E10" t="str">
-        <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
       </c>
       <c r="F10" t="str">
-        <v>Ремонт и тюнинг фар DODGE в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар FERRARI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G10" t="str">
-        <v>ремонт фар dodge, ремонт фар dodge спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар ferrari, ремонт фар ferrari спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H10" t="str">
-        <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
       </c>
       <c r="I10" t="str">
-        <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>FERRARI</v>
+        <v>FORD</v>
       </c>
       <c r="B11" t="str">
-        <v>ferrari</v>
+        <v>ford</v>
       </c>
       <c r="C11" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ferrari-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-ford_motor_company_logo.svg.png</v>
       </c>
       <c r="D11" t="str">
-        <v>ремонт фар ferrari</v>
+        <v>ремонт фар ford</v>
       </c>
       <c r="E11" t="str">
-        <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
       </c>
       <c r="F11" t="str">
-        <v>Ремонт и тюнинг фар FERRARI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар FORD в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G11" t="str">
-        <v>ремонт фар ferrari, ремонт фар ferrari спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар ford, ремонт фар ford спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H11" t="str">
-        <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
       </c>
       <c r="I11" t="str">
-        <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>FORD</v>
+        <v>HONDA</v>
       </c>
       <c r="B12" t="str">
-        <v>ford</v>
+        <v>honda</v>
       </c>
       <c r="C12" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-ford_motor_company_logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/honda.webp</v>
       </c>
       <c r="D12" t="str">
-        <v>ремонт фар ford</v>
+        <v>ремонт фар honda</v>
       </c>
       <c r="E12" t="str">
-        <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
       </c>
       <c r="F12" t="str">
-        <v>Ремонт и тюнинг фар FORD в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар HONDA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G12" t="str">
-        <v>ремонт фар ford, ремонт фар ford спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар honda, ремонт фар honda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H12" t="str">
-        <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
       </c>
       <c r="I12" t="str">
-        <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>HONDA</v>
+        <v>HUMMER</v>
       </c>
       <c r="B13" t="str">
-        <v>honda</v>
+        <v>hummer</v>
       </c>
       <c r="C13" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-honda.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-hummer.svg.png</v>
       </c>
       <c r="D13" t="str">
-        <v>ремонт фар honda</v>
+        <v>ремонт фар hummer</v>
       </c>
       <c r="E13" t="str">
-        <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
       </c>
       <c r="F13" t="str">
-        <v>Ремонт и тюнинг фар HONDA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар HUMMER в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G13" t="str">
-        <v>ремонт фар honda, ремонт фар honda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар hummer, ремонт фар hummer спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H13" t="str">
-        <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
       </c>
       <c r="I13" t="str">
-        <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>HPL</v>
+        <v>Hyundai</v>
       </c>
       <c r="B14" t="str">
-        <v>hpl</v>
+        <v>hyundai</v>
       </c>
       <c r="C14" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-incandescent_light_bulb.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/hyundai.svg</v>
       </c>
       <c r="D14" t="str">
-        <v>ремонт фар hpl</v>
+        <v>ремонт фар hyundai</v>
       </c>
       <c r="E14" t="str">
-        <v>Ремонт и тюнинг фар HPL в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
       </c>
       <c r="F14" t="str">
-        <v>Ремонт и тюнинг фар HPL в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар Hyundai в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G14" t="str">
-        <v>ремонт фар hpl, ремонт фар hpl спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар hyundai, ремонт фар hyundai спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H14" t="str">
-        <v>Ремонт и тюнинг фар HPL в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
       </c>
       <c r="I14" t="str">
-        <v>Ремонт и тюнинг фар HPL в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>HUMMER</v>
+        <v>INFINITI</v>
       </c>
       <c r="B15" t="str">
-        <v>hummer</v>
+        <v>infiniti</v>
       </c>
       <c r="C15" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-hummer.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/infiniti-logo.png</v>
       </c>
       <c r="D15" t="str">
-        <v>ремонт фар hummer</v>
+        <v>ремонт фар infiniti</v>
       </c>
       <c r="E15" t="str">
-        <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
       </c>
       <c r="F15" t="str">
-        <v>Ремонт и тюнинг фар HUMMER в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар INFINITI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G15" t="str">
-        <v>ремонт фар hummer, ремонт фар hummer спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар infiniti, ремонт фар infiniti спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H15" t="str">
-        <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
       </c>
       <c r="I15" t="str">
-        <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Hyundai</v>
+        <v>JAGUAR</v>
       </c>
       <c r="B16" t="str">
-        <v>hyundai</v>
+        <v>jaguar</v>
       </c>
       <c r="C16" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-hyundai_motor_company_logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/jaguar-logo.png</v>
       </c>
       <c r="D16" t="str">
-        <v>ремонт фар hyundai</v>
+        <v>ремонт фар jaguar</v>
       </c>
       <c r="E16" t="str">
-        <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
       </c>
       <c r="F16" t="str">
-        <v>Ремонт и тюнинг фар Hyundai в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар JAGUAR в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G16" t="str">
-        <v>ремонт фар hyundai, ремонт фар hyundai спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар jaguar, ремонт фар jaguar спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H16" t="str">
-        <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
       </c>
       <c r="I16" t="str">
-        <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>INFINITI</v>
+        <v>JEEP</v>
       </c>
       <c r="B17" t="str">
-        <v>infiniti</v>
+        <v>jeep</v>
       </c>
       <c r="C17" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/infiniti-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-jeep_logo.svg.png</v>
       </c>
       <c r="D17" t="str">
-        <v>ремонт фар infiniti</v>
+        <v>ремонт фар jeep</v>
       </c>
       <c r="E17" t="str">
-        <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
       </c>
       <c r="F17" t="str">
-        <v>Ремонт и тюнинг фар INFINITI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар JEEP в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G17" t="str">
-        <v>ремонт фар infiniti, ремонт фар infiniti спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар jeep, ремонт фар jeep спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H17" t="str">
-        <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
       </c>
       <c r="I17" t="str">
-        <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>JAGUAR</v>
+        <v>KIA</v>
       </c>
       <c r="B18" t="str">
-        <v>jaguar</v>
+        <v>kia</v>
       </c>
       <c r="C18" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/jaguar-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/kia.webp</v>
       </c>
       <c r="D18" t="str">
-        <v>ремонт фар jaguar</v>
+        <v>ремонт фар kia</v>
       </c>
       <c r="E18" t="str">
-        <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
       </c>
       <c r="F18" t="str">
-        <v>Ремонт и тюнинг фар JAGUAR в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар KIA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G18" t="str">
-        <v>ремонт фар jaguar, ремонт фар jaguar спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар kia, ремонт фар kia спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H18" t="str">
-        <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
       </c>
       <c r="I18" t="str">
-        <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>JEEP</v>
+        <v>KTM</v>
       </c>
       <c r="B19" t="str">
-        <v>jeep</v>
+        <v>ktm</v>
       </c>
       <c r="C19" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-jeep_logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ktm.svg</v>
       </c>
       <c r="D19" t="str">
-        <v>ремонт фар jeep</v>
+        <v>ремонт фар ktm</v>
       </c>
       <c r="E19" t="str">
-        <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
       </c>
       <c r="F19" t="str">
-        <v>Ремонт и тюнинг фар JEEP в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар KTM в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G19" t="str">
-        <v>ремонт фар jeep, ремонт фар jeep спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар ktm, ремонт фар ktm спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H19" t="str">
-        <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
       </c>
       <c r="I19" t="str">
-        <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>KIA</v>
+        <v>Land Rover</v>
       </c>
       <c r="B20" t="str">
-        <v>kia</v>
+        <v>land-rover</v>
       </c>
       <c r="C20" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-kia_logo3.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/land-rover.svg</v>
       </c>
       <c r="D20" t="str">
-        <v>ремонт фар kia</v>
+        <v>ремонт фар land rover</v>
       </c>
       <c r="E20" t="str">
-        <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
       </c>
       <c r="F20" t="str">
-        <v>Ремонт и тюнинг фар KIA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар Land Rover в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G20" t="str">
-        <v>ремонт фар kia, ремонт фар kia спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар land rover, ремонт фар land rover спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H20" t="str">
-        <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
       </c>
       <c r="I20" t="str">
-        <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>KTM</v>
+        <v>LEXUS</v>
       </c>
       <c r="B21" t="str">
-        <v>ktm</v>
+        <v>lexus</v>
       </c>
       <c r="C21" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-ktm-logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/lexus.webp</v>
       </c>
       <c r="D21" t="str">
-        <v>ремонт фар ktm</v>
+        <v>ремонт фар lexus</v>
       </c>
       <c r="E21" t="str">
-        <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
       </c>
       <c r="F21" t="str">
-        <v>Ремонт и тюнинг фар KTM в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар LEXUS в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G21" t="str">
-        <v>ремонт фар ktm, ремонт фар ktm спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар lexus, ремонт фар lexus спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H21" t="str">
-        <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
       </c>
       <c r="I21" t="str">
-        <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Land Rover</v>
+        <v>Maserati</v>
       </c>
       <c r="B22" t="str">
-        <v>land-rover</v>
+        <v>maserati</v>
       </c>
       <c r="C22" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/land-rover-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/maserati_logo.svg</v>
       </c>
       <c r="D22" t="str">
-        <v>ремонт фар land rover</v>
+        <v>ремонт фар maserati</v>
       </c>
       <c r="E22" t="str">
-        <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
       </c>
       <c r="F22" t="str">
-        <v>Ремонт и тюнинг фар Land Rover в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар Maserati в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G22" t="str">
-        <v>ремонт фар land rover, ремонт фар land rover спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар maserati, ремонт фар maserati спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H22" t="str">
-        <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
       </c>
       <c r="I22" t="str">
-        <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>LEXUS</v>
+        <v>Maybach</v>
       </c>
       <c r="B23" t="str">
-        <v>lexus</v>
+        <v>maybach</v>
       </c>
       <c r="C23" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/lexus-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/maybach.svg</v>
       </c>
       <c r="D23" t="str">
-        <v>ремонт фар lexus</v>
+        <v>ремонт фар maybach</v>
       </c>
       <c r="E23" t="str">
-        <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
       </c>
       <c r="F23" t="str">
-        <v>Ремонт и тюнинг фар LEXUS в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар Maybach в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G23" t="str">
-        <v>ремонт фар lexus, ремонт фар lexus спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар maybach, ремонт фар maybach спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H23" t="str">
-        <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
       </c>
       <c r="I23" t="str">
-        <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Maserati</v>
+        <v>MAZDA</v>
       </c>
       <c r="B24" t="str">
-        <v>maserati</v>
+        <v>mazda</v>
       </c>
       <c r="C24" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/maserati-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mazda.svg</v>
       </c>
       <c r="D24" t="str">
-        <v>ремонт фар maserati</v>
+        <v>ремонт фар mazda</v>
       </c>
       <c r="E24" t="str">
-        <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
       </c>
       <c r="F24" t="str">
-        <v>Ремонт и тюнинг фар Maserati в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар MAZDA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G24" t="str">
-        <v>ремонт фар maserati, ремонт фар maserati спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар mazda, ремонт фар mazda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H24" t="str">
-        <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
       </c>
       <c r="I24" t="str">
-        <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Maybach</v>
+        <v>MERCEDES</v>
       </c>
       <c r="B25" t="str">
-        <v>maybach</v>
+        <v>mercedes</v>
       </c>
       <c r="C25" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-maybach-logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mercedes.webp</v>
       </c>
       <c r="D25" t="str">
-        <v>ремонт фар maybach</v>
+        <v>ремонт фар mercedes</v>
       </c>
       <c r="E25" t="str">
-        <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
       </c>
       <c r="F25" t="str">
-        <v>Ремонт и тюнинг фар Maybach в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар MERCEDES в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G25" t="str">
-        <v>ремонт фар maybach, ремонт фар maybach спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар mercedes, ремонт фар mercedes спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H25" t="str">
-        <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
       </c>
       <c r="I25" t="str">
-        <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MAZDA</v>
+        <v>MINI</v>
       </c>
       <c r="B26" t="str">
-        <v>mazda</v>
+        <v>mini</v>
       </c>
       <c r="C26" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mazda-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mini-logo.png</v>
       </c>
       <c r="D26" t="str">
-        <v>ремонт фар mazda</v>
+        <v>ремонт фар mini</v>
       </c>
       <c r="E26" t="str">
-        <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
       </c>
       <c r="F26" t="str">
-        <v>Ремонт и тюнинг фар MAZDA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар MINI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G26" t="str">
-        <v>ремонт фар mazda, ремонт фар mazda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар mini, ремонт фар mini спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H26" t="str">
-        <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
       </c>
       <c r="I26" t="str">
-        <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>MERCEDES</v>
+        <v>MITSUBISHI</v>
       </c>
       <c r="B27" t="str">
-        <v>mercedes</v>
+        <v>mitsubishi</v>
       </c>
       <c r="C27" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mercedes-benz-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mitsubishi.svg</v>
       </c>
       <c r="D27" t="str">
-        <v>ремонт фар mercedes</v>
+        <v>ремонт фар mitsubishi</v>
       </c>
       <c r="E27" t="str">
-        <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
       </c>
       <c r="F27" t="str">
-        <v>Ремонт и тюнинг фар MERCEDES в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар MITSUBISHI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G27" t="str">
-        <v>ремонт фар mercedes, ремонт фар mercedes спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар mitsubishi, ремонт фар mitsubishi спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H27" t="str">
-        <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
       </c>
       <c r="I27" t="str">
-        <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MINI</v>
+        <v>NISSAN</v>
       </c>
       <c r="B28" t="str">
-        <v>mini</v>
+        <v>nissan</v>
       </c>
       <c r="C28" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mini-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-nissan_logo.svg.png</v>
       </c>
       <c r="D28" t="str">
-        <v>ремонт фар mini</v>
+        <v>ремонт фар nissan</v>
       </c>
       <c r="E28" t="str">
-        <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
       </c>
       <c r="F28" t="str">
-        <v>Ремонт и тюнинг фар MINI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар NISSAN в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G28" t="str">
-        <v>ремонт фар mini, ремонт фар mini спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар nissan, ремонт фар nissan спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H28" t="str">
-        <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
       </c>
       <c r="I28" t="str">
-        <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MITSUBISHI</v>
+        <v>OPEL</v>
       </c>
       <c r="B29" t="str">
-        <v>mitsubishi</v>
+        <v>opel</v>
       </c>
       <c r="C29" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-mitsubishi_logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/opel.svg</v>
       </c>
       <c r="D29" t="str">
-        <v>ремонт фар mitsubishi</v>
+        <v>ремонт фар opel</v>
       </c>
       <c r="E29" t="str">
-        <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
       </c>
       <c r="F29" t="str">
-        <v>Ремонт и тюнинг фар MITSUBISHI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар OPEL в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G29" t="str">
-        <v>ремонт фар mitsubishi, ремонт фар mitsubishi спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар opel, ремонт фар opel спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H29" t="str">
-        <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
       </c>
       <c r="I29" t="str">
-        <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>NISSAN</v>
+        <v>PEUGEOT</v>
       </c>
       <c r="B30" t="str">
-        <v>nissan</v>
+        <v>peugeot</v>
       </c>
       <c r="C30" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-nissan_logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/peugeot.svg</v>
       </c>
       <c r="D30" t="str">
-        <v>ремонт фар nissan</v>
+        <v>ремонт фар peugeot</v>
       </c>
       <c r="E30" t="str">
-        <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
       </c>
       <c r="F30" t="str">
-        <v>Ремонт и тюнинг фар NISSAN в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар PEUGEOT в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G30" t="str">
-        <v>ремонт фар nissan, ремонт фар nissan спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар peugeot, ремонт фар peugeot спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H30" t="str">
-        <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
       </c>
       <c r="I30" t="str">
-        <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>OPEL</v>
+        <v>PORSCHE</v>
       </c>
       <c r="B31" t="str">
-        <v>opel</v>
+        <v>porsche</v>
       </c>
       <c r="C31" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-opel_logo_2023.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/porsche-logo.png</v>
       </c>
       <c r="D31" t="str">
-        <v>ремонт фар opel</v>
+        <v>ремонт фар porsche</v>
       </c>
       <c r="E31" t="str">
-        <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
       </c>
       <c r="F31" t="str">
-        <v>Ремонт и тюнинг фар OPEL в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар PORSCHE в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G31" t="str">
-        <v>ремонт фар opel, ремонт фар opel спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар porsche, ремонт фар porsche спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H31" t="str">
-        <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
       </c>
       <c r="I31" t="str">
-        <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>PEUGEOT</v>
+        <v>RENAULT</v>
       </c>
       <c r="B32" t="str">
-        <v>peugeot</v>
+        <v>renault</v>
       </c>
       <c r="C32" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/peugeot-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/renault-logo.png</v>
       </c>
       <c r="D32" t="str">
-        <v>ремонт фар peugeot</v>
+        <v>ремонт фар renault</v>
       </c>
       <c r="E32" t="str">
-        <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
       </c>
       <c r="F32" t="str">
-        <v>Ремонт и тюнинг фар PEUGEOT в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар RENAULT в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G32" t="str">
-        <v>ремонт фар peugeot, ремонт фар peugeot спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар renault, ремонт фар renault спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H32" t="str">
-        <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
       </c>
       <c r="I32" t="str">
-        <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>PORSCHE</v>
+        <v>Rolls-Royce</v>
       </c>
       <c r="B33" t="str">
-        <v>porsche</v>
+        <v>rolls-royce</v>
       </c>
       <c r="C33" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/porsche-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-rolls-royce_motor_cars_logo.svg.png</v>
       </c>
       <c r="D33" t="str">
-        <v>ремонт фар porsche</v>
+        <v>ремонт фар rolls-royce</v>
       </c>
       <c r="E33" t="str">
-        <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
       </c>
       <c r="F33" t="str">
-        <v>Ремонт и тюнинг фар PORSCHE в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар Rolls-Royce в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G33" t="str">
-        <v>ремонт фар porsche, ремонт фар porsche спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар rolls-royce, ремонт фар rolls-royce спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H33" t="str">
-        <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
       </c>
       <c r="I33" t="str">
-        <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>RENAULT</v>
+        <v>SAAB</v>
       </c>
       <c r="B34" t="str">
-        <v>renault</v>
+        <v>saab</v>
       </c>
       <c r="C34" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/renault-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/saab.svg</v>
       </c>
       <c r="D34" t="str">
-        <v>ремонт фар renault</v>
+        <v>ремонт фар saab</v>
       </c>
       <c r="E34" t="str">
-        <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
       </c>
       <c r="F34" t="str">
-        <v>Ремонт и тюнинг фар RENAULT в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар SAAB в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G34" t="str">
-        <v>ремонт фар renault, ремонт фар renault спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар saab, ремонт фар saab спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H34" t="str">
-        <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
       </c>
       <c r="I34" t="str">
-        <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Rolls-Royce</v>
+        <v>Skoda</v>
       </c>
       <c r="B35" t="str">
-        <v>rolls-royce</v>
+        <v>skoda</v>
       </c>
       <c r="C35" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-rolls-royce_motor_cars_logo.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/skoda.svg</v>
       </c>
       <c r="D35" t="str">
-        <v>ремонт фар rolls-royce</v>
+        <v>ремонт фар skoda</v>
       </c>
       <c r="E35" t="str">
-        <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
       </c>
       <c r="F35" t="str">
-        <v>Ремонт и тюнинг фар Rolls-Royce в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар Skoda в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G35" t="str">
-        <v>ремонт фар rolls-royce, ремонт фар rolls-royce спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар skoda, ремонт фар skoda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H35" t="str">
-        <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
       </c>
       <c r="I35" t="str">
-        <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>SAAB</v>
+        <v>SsangYong</v>
       </c>
       <c r="B36" t="str">
-        <v>saab</v>
+        <v>ssangyong</v>
       </c>
       <c r="C36" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/saab-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ssangyong-logo.png</v>
       </c>
       <c r="D36" t="str">
-        <v>ремонт фар saab</v>
+        <v>ремонт фар ssangyong</v>
       </c>
       <c r="E36" t="str">
-        <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
       </c>
       <c r="F36" t="str">
-        <v>Ремонт и тюнинг фар SAAB в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар SsangYong в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G36" t="str">
-        <v>ремонт фар saab, ремонт фар saab спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар ssangyong, ремонт фар ssangyong спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H36" t="str">
-        <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
       </c>
       <c r="I36" t="str">
-        <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Skoda</v>
+        <v>SUBARU</v>
       </c>
       <c r="B37" t="str">
-        <v>skoda</v>
+        <v>subaru</v>
       </c>
       <c r="C37" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/skoda-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/subaru-logo.png</v>
       </c>
       <c r="D37" t="str">
-        <v>ремонт фар skoda</v>
+        <v>ремонт фар subaru</v>
       </c>
       <c r="E37" t="str">
-        <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
       </c>
       <c r="F37" t="str">
-        <v>Ремонт и тюнинг фар Skoda в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар SUBARU в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G37" t="str">
-        <v>ремонт фар skoda, ремонт фар skoda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар subaru, ремонт фар subaru спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H37" t="str">
-        <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
       </c>
       <c r="I37" t="str">
-        <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>SsangYong</v>
+        <v>SUZUKI</v>
       </c>
       <c r="B38" t="str">
-        <v>ssangyong</v>
+        <v>suzuki</v>
       </c>
       <c r="C38" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ssangyong-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/suzuki.svg</v>
       </c>
       <c r="D38" t="str">
-        <v>ремонт фар ssangyong</v>
+        <v>ремонт фар suzuki</v>
       </c>
       <c r="E38" t="str">
-        <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
       </c>
       <c r="F38" t="str">
-        <v>Ремонт и тюнинг фар SsangYong в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар SUZUKI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G38" t="str">
-        <v>ремонт фар ssangyong, ремонт фар ssangyong спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар suzuki, ремонт фар suzuki спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H38" t="str">
-        <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
       </c>
       <c r="I38" t="str">
-        <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>SUBARU</v>
+        <v>TOYOTA</v>
       </c>
       <c r="B39" t="str">
-        <v>subaru</v>
+        <v>toyota</v>
       </c>
       <c r="C39" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/subaru-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/toyota.webp</v>
       </c>
       <c r="D39" t="str">
-        <v>ремонт фар subaru</v>
+        <v>ремонт фар toyota</v>
       </c>
       <c r="E39" t="str">
-        <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
       </c>
       <c r="F39" t="str">
-        <v>Ремонт и тюнинг фар SUBARU в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар TOYOTA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G39" t="str">
-        <v>ремонт фар subaru, ремонт фар subaru спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар toyota, ремонт фар toyota спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H39" t="str">
-        <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
       </c>
       <c r="I39" t="str">
-        <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>SUZUKI</v>
+        <v>Volkswagen</v>
       </c>
       <c r="B40" t="str">
-        <v>suzuki</v>
+        <v>vw</v>
       </c>
       <c r="C40" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/suzuki-logo.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/volkswagen.webp</v>
       </c>
       <c r="D40" t="str">
-        <v>ремонт фар suzuki</v>
+        <v>ремонт фар volkswagen</v>
       </c>
       <c r="E40" t="str">
-        <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
       </c>
       <c r="F40" t="str">
-        <v>Ремонт и тюнинг фар SUZUKI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар Volkswagen в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G40" t="str">
-        <v>ремонт фар suzuki, ремонт фар suzuki спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар volkswagen, ремонт фар volkswagen спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H40" t="str">
-        <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
       </c>
       <c r="I40" t="str">
-        <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>TOYOTA</v>
+        <v>VOLVO</v>
       </c>
       <c r="B41" t="str">
-        <v>toyota</v>
+        <v>volvo</v>
       </c>
       <c r="C41" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-toyota.svg.png</v>
+        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/volvo.svg</v>
       </c>
       <c r="D41" t="str">
-        <v>ремонт фар toyota</v>
+        <v>ремонт фар volvo</v>
       </c>
       <c r="E41" t="str">
-        <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар VOLVO в СПб | КБ АВТО</v>
       </c>
       <c r="F41" t="str">
-        <v>Ремонт и тюнинг фар TOYOTA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+        <v>Ремонт и тюнинг фар VOLVO в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
       </c>
       <c r="G41" t="str">
-        <v>ремонт фар toyota, ремонт фар toyota спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+        <v>ремонт фар volvo, ремонт фар volvo спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H41" t="str">
-        <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
+        <v>Ремонт и тюнинг фар VOLVO в СПб | КБ АВТО</v>
       </c>
       <c r="I41" t="str">
-        <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>Volkswagen</v>
-      </c>
-      <c r="B42" t="str">
-        <v>vw</v>
-      </c>
-      <c r="C42" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-volkswagen_logo_2019.svg.png</v>
-      </c>
-      <c r="D42" t="str">
-        <v>ремонт фар volkswagen</v>
-      </c>
-      <c r="E42" t="str">
-        <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
-      </c>
-      <c r="F42" t="str">
-        <v>Ремонт и тюнинг фар Volkswagen в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G42" t="str">
-        <v>ремонт фар volkswagen, ремонт фар volkswagen спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
-      </c>
-      <c r="H42" t="str">
-        <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
-      </c>
-      <c r="I42" t="str">
-        <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>VOLVO</v>
-      </c>
-      <c r="B43" t="str">
-        <v>volvo</v>
-      </c>
-      <c r="C43" t="str">
-        <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-volvo_logo.svg.png</v>
-      </c>
-      <c r="D43" t="str">
-        <v>ремонт фар volvo</v>
-      </c>
-      <c r="E43" t="str">
-        <v>Ремонт и тюнинг фар VOLVO в СПб | КБ АВТО</v>
-      </c>
-      <c r="F43" t="str">
-        <v>Ремонт и тюнинг фар VOLVO в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G43" t="str">
-        <v>ремонт фар volvo, ремонт фар volvo спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
-      </c>
-      <c r="H43" t="str">
-        <v>Ремонт и тюнинг фар VOLVO в СПб | КБ АВТО</v>
-      </c>
-      <c r="I43" t="str">
         <v>Ремонт и тюнинг фар VOLVO в СПб | КБ АВТО</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update single brand page
</commit_message>
<xml_diff>
--- a/parsing/data/brands-import.xlsx
+++ b/parsing/data/brands-import.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:L41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,21 +410,30 @@
         <v>image</v>
       </c>
       <c r="D1" t="str">
+        <v>hero_title</v>
+      </c>
+      <c r="E1" t="str">
+        <v>features_title</v>
+      </c>
+      <c r="F1" t="str">
+        <v>features</v>
+      </c>
+      <c r="G1" t="str">
         <v>Focus Keyword</v>
       </c>
-      <c r="E1" t="str">
+      <c r="H1" t="str">
         <v>SEO Title</v>
       </c>
-      <c r="F1" t="str">
+      <c r="I1" t="str">
         <v>Meta Description</v>
       </c>
-      <c r="G1" t="str">
+      <c r="J1" t="str">
         <v>Meta Keywords</v>
       </c>
-      <c r="H1" t="str">
+      <c r="K1" t="str">
         <v>Facebook Title</v>
       </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>Twitter Title</v>
       </c>
     </row>
@@ -439,21 +448,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/acura.svg</v>
       </c>
       <c r="D2" t="str">
+        <v>Ремонт фар ACURA</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Особенности ремонта фар ACURA</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Герметизация и «стекло»::Фары ACURA из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На ACURA светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар ACURA чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары ACURA собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G2" t="str">
         <v>ремонт фар acura</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Ремонт и тюнинг фар ACURA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G2" t="str">
-        <v>ремонт фар acura, ремонт фар acura спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H2" t="str">
         <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
       </c>
       <c r="I2" t="str">
+        <v>Ремонт и тюнинг фар ACURA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J2" t="str">
+        <v>ремонт фар acura, ремонт фар acura спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
+      </c>
+      <c r="L2" t="str">
         <v>Ремонт и тюнинг фар ACURA в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -468,21 +486,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/audi-logo.svg</v>
       </c>
       <c r="D3" t="str">
+        <v>Ремонт фар AUDI</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Особенности ремонта фар AUDI</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Матричный свет и Matrix LED::На Audi (A6 C7/C8, A8, Q7/Q8) часто выгорают отдельные сегменты Matrix LED и блоки управления. Простая замена лампы не поможет — нужна диагностика шины, прошивка и точечный ремонт драйверов.|Герметизация и стёкла::Поликарбонатные стёкла Audi мутнеют и желтеют. Заводской лак тонкий: грубая полировка снимает УФ-защиту. Корректный ремонт — снятие лака, шлифовка и новый двухкомпонентный защитный слой.|Запотевание и дренаж::Вентиляционные мембраны в корпусах Audi часто забиваются. Если загерметизировать шов без замены дренажа, внутри скапливается конденсат — «аквариум» и коррозия контактов.|Разбор корпуса и линзы::Современные фары Audi собраны на жёстком герметике. Вскрытие только с контролем температуры. Замена линз или LED-модулей требует аккуратной пайки и калибровки светотеневой границы.</v>
+      </c>
+      <c r="G3" t="str">
         <v>ремонт фар audi</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Ремонт и тюнинг фар AUDI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G3" t="str">
-        <v>ремонт фар audi, ремонт фар audi спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H3" t="str">
         <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
       </c>
       <c r="I3" t="str">
+        <v>Ремонт и тюнинг фар AUDI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J3" t="str">
+        <v>ремонт фар audi, ремонт фар audi спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
+      </c>
+      <c r="L3" t="str">
         <v>Ремонт и тюнинг фар AUDI в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -497,21 +524,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/bentley_logo.svg</v>
       </c>
       <c r="D4" t="str">
+        <v>Ремонт фар BENTLEY</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Особенности ремонта фар BENTLEY</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Герметизация и «стекло»::Фары BENTLEY из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На BENTLEY светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар BENTLEY чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары BENTLEY собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G4" t="str">
         <v>ремонт фар bentley</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Ремонт и тюнинг фар BENTLEY в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G4" t="str">
-        <v>ремонт фар bentley, ремонт фар bentley спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H4" t="str">
         <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
       </c>
       <c r="I4" t="str">
+        <v>Ремонт и тюнинг фар BENTLEY в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J4" t="str">
+        <v>ремонт фар bentley, ремонт фар bentley спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
+      </c>
+      <c r="L4" t="str">
         <v>Ремонт и тюнинг фар BENTLEY в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -526,21 +562,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/bmw.svg</v>
       </c>
       <c r="D5" t="str">
+        <v>Ремонт фар BMW</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Особенности ремонта фар BMW</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Герметизация и «стекло»::Фары BMW из поликарбоната мутнеют и царапаются. Заводской лак на них очень твердый, но тонкий. Грубая полировка стирает УФ-защиту навсегда. Правильный ремонт — это полное снятие старого лака, глубокая шлифовка и нанесение нового двухкомпонентного защитного слоя.|Электроника и датчики::Просто заменить диод нельзя. Светодиодные фары плотно интегрированы с блоками TMS, которые горят при замыкании или сырости. Часто проблема в сгоревших драйверах на плате. Ремонт требует микроэлектроники: диагностики, пайки шлейфов и чистки под микроскопом.|Разгерметизация и дренаж::Корпуса имеют сложную вентиляцию с мембранами, а не просто заглушки. Запотевание почти всегда вызвано забитыми или разрушенными мембранами, а не только трещинами. Если просто залить шов герметиком, не заменив мембраны, фара превратится в «аквариум».|Неразборный корпус и линзы::Современные модели (G-серия, лазерный свет) собраны на жестком полиуретановом герметике. Вскрытие требует точного нагрева или аккуратного распила шва. Кустарный разбор ведет к трещинам дорогого пластика. Замена битых линз или LED-модулей — это ювелирная пайка на едином радиаторе.</v>
+      </c>
+      <c r="G5" t="str">
         <v>ремонт фар bmw</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Ремонт и тюнинг фар BMW в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G5" t="str">
-        <v>ремонт фар bmw, ремонт фар bmw спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H5" t="str">
         <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
       </c>
       <c r="I5" t="str">
+        <v>Ремонт и тюнинг фар BMW в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J5" t="str">
+        <v>ремонт фар bmw, ремонт фар bmw спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
+      </c>
+      <c r="L5" t="str">
         <v>Ремонт и тюнинг фар BMW в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -555,21 +600,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/cadillac.svg</v>
       </c>
       <c r="D6" t="str">
+        <v>Ремонт фар CADILLAC</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Особенности ремонта фар CADILLAC</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Герметизация и «стекло»::Фары CADILLAC из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На CADILLAC светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар CADILLAC чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары CADILLAC собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G6" t="str">
         <v>ремонт фар cadillac</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Ремонт и тюнинг фар CADILLAC в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G6" t="str">
-        <v>ремонт фар cadillac, ремонт фар cadillac спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H6" t="str">
         <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
       </c>
       <c r="I6" t="str">
+        <v>Ремонт и тюнинг фар CADILLAC в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J6" t="str">
+        <v>ремонт фар cadillac, ремонт фар cadillac спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
+      </c>
+      <c r="L6" t="str">
         <v>Ремонт и тюнинг фар CADILLAC в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -584,21 +638,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/chevrolet.webp</v>
       </c>
       <c r="D7" t="str">
+        <v>Ремонт фар CHEVROLET</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Особенности ремонта фар CHEVROLET</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Герметизация и «стекло»::Фары CHEVROLET из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На CHEVROLET светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар CHEVROLET чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары CHEVROLET собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G7" t="str">
         <v>ремонт фар chevrolet</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Ремонт и тюнинг фар CHEVROLET в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G7" t="str">
-        <v>ремонт фар chevrolet, ремонт фар chevrolet спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H7" t="str">
         <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
       </c>
       <c r="I7" t="str">
+        <v>Ремонт и тюнинг фар CHEVROLET в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J7" t="str">
+        <v>ремонт фар chevrolet, ремонт фар chevrolet спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
+      </c>
+      <c r="L7" t="str">
         <v>Ремонт и тюнинг фар CHEVROLET в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -613,21 +676,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-chryply_blue_pentastar.svg.png</v>
       </c>
       <c r="D8" t="str">
+        <v>Ремонт фар CHRYSLER</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Особенности ремонта фар CHRYSLER</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Герметизация и «стекло»::Фары CHRYSLER из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На CHRYSLER светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар CHRYSLER чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары CHRYSLER собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G8" t="str">
         <v>ремонт фар chrysler</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Ремонт и тюнинг фар CHRYSLER в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G8" t="str">
-        <v>ремонт фар chrysler, ремонт фар chrysler спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H8" t="str">
         <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
       </c>
       <c r="I8" t="str">
+        <v>Ремонт и тюнинг фар CHRYSLER в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J8" t="str">
+        <v>ремонт фар chrysler, ремонт фар chrysler спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
+      </c>
+      <c r="L8" t="str">
         <v>Ремонт и тюнинг фар CHRYSLER в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -642,21 +714,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/dodge.svg</v>
       </c>
       <c r="D9" t="str">
+        <v>Ремонт фар DODGE</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Особенности ремонта фар DODGE</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Герметизация и «стекло»::Фары DODGE из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На DODGE светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар DODGE чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары DODGE собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G9" t="str">
         <v>ремонт фар dodge</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Ремонт и тюнинг фар DODGE в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G9" t="str">
-        <v>ремонт фар dodge, ремонт фар dodge спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H9" t="str">
         <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
       </c>
       <c r="I9" t="str">
+        <v>Ремонт и тюнинг фар DODGE в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J9" t="str">
+        <v>ремонт фар dodge, ремонт фар dodge спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
+      </c>
+      <c r="L9" t="str">
         <v>Ремонт и тюнинг фар DODGE в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -671,21 +752,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ferrari-logo.png</v>
       </c>
       <c r="D10" t="str">
+        <v>Ремонт фар FERRARI</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Особенности ремонта фар FERRARI</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Герметизация и «стекло»::Фары FERRARI из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На FERRARI светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар FERRARI чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары FERRARI собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G10" t="str">
         <v>ремонт фар ferrari</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Ремонт и тюнинг фар FERRARI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G10" t="str">
-        <v>ремонт фар ferrari, ремонт фар ferrari спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H10" t="str">
         <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
       </c>
       <c r="I10" t="str">
+        <v>Ремонт и тюнинг фар FERRARI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J10" t="str">
+        <v>ремонт фар ferrari, ремонт фар ferrari спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
+      </c>
+      <c r="L10" t="str">
         <v>Ремонт и тюнинг фар FERRARI в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -700,21 +790,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-ford_motor_company_logo.svg.png</v>
       </c>
       <c r="D11" t="str">
+        <v>Ремонт фар FORD</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Особенности ремонта фар FORD</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Герметизация и «стекло»::Фары FORD из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На FORD светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар FORD чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары FORD собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G11" t="str">
         <v>ремонт фар ford</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Ремонт и тюнинг фар FORD в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G11" t="str">
-        <v>ремонт фар ford, ремонт фар ford спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H11" t="str">
         <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
       </c>
       <c r="I11" t="str">
+        <v>Ремонт и тюнинг фар FORD в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J11" t="str">
+        <v>ремонт фар ford, ремонт фар ford спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
+      </c>
+      <c r="L11" t="str">
         <v>Ремонт и тюнинг фар FORD в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -729,21 +828,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/honda.webp</v>
       </c>
       <c r="D12" t="str">
+        <v>Ремонт фар HONDA</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Особенности ремонта фар HONDA</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Герметизация и «стекло»::Фары HONDA из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На HONDA светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар HONDA чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары HONDA собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G12" t="str">
         <v>ремонт фар honda</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Ремонт и тюнинг фар HONDA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G12" t="str">
-        <v>ремонт фар honda, ремонт фар honda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H12" t="str">
         <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
       </c>
       <c r="I12" t="str">
+        <v>Ремонт и тюнинг фар HONDA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J12" t="str">
+        <v>ремонт фар honda, ремонт фар honda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
+      </c>
+      <c r="L12" t="str">
         <v>Ремонт и тюнинг фар HONDA в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -758,21 +866,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-hummer.svg.png</v>
       </c>
       <c r="D13" t="str">
+        <v>Ремонт фар HUMMER</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Особенности ремонта фар HUMMER</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Герметизация и «стекло»::Фары HUMMER из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На HUMMER светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар HUMMER чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары HUMMER собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G13" t="str">
         <v>ремонт фар hummer</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Ремонт и тюнинг фар HUMMER в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G13" t="str">
-        <v>ремонт фар hummer, ремонт фар hummer спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H13" t="str">
         <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
       </c>
       <c r="I13" t="str">
+        <v>Ремонт и тюнинг фар HUMMER в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J13" t="str">
+        <v>ремонт фар hummer, ремонт фар hummer спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
+      </c>
+      <c r="L13" t="str">
         <v>Ремонт и тюнинг фар HUMMER в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -787,21 +904,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/hyundai.svg</v>
       </c>
       <c r="D14" t="str">
+        <v>Ремонт фар Hyundai</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Особенности ремонта фар Hyundai</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Герметизация и «стекло»::Фары Hyundai из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На Hyundai светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар Hyundai чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары Hyundai собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G14" t="str">
         <v>ремонт фар hyundai</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Ремонт и тюнинг фар Hyundai в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G14" t="str">
-        <v>ремонт фар hyundai, ремонт фар hyundai спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H14" t="str">
         <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
       </c>
       <c r="I14" t="str">
+        <v>Ремонт и тюнинг фар Hyundai в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J14" t="str">
+        <v>ремонт фар hyundai, ремонт фар hyundai спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
+      </c>
+      <c r="L14" t="str">
         <v>Ремонт и тюнинг фар Hyundai в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -816,21 +942,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/infiniti-logo.png</v>
       </c>
       <c r="D15" t="str">
+        <v>Ремонт фар INFINITI</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Особенности ремонта фар INFINITI</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Герметизация и «стекло»::Фары INFINITI из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На INFINITI светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар INFINITI чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары INFINITI собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G15" t="str">
         <v>ремонт фар infiniti</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Ремонт и тюнинг фар INFINITI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G15" t="str">
-        <v>ремонт фар infiniti, ремонт фар infiniti спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H15" t="str">
         <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
       </c>
       <c r="I15" t="str">
+        <v>Ремонт и тюнинг фар INFINITI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J15" t="str">
+        <v>ремонт фар infiniti, ремонт фар infiniti спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
+      </c>
+      <c r="L15" t="str">
         <v>Ремонт и тюнинг фар INFINITI в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -845,21 +980,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/jaguar-logo.png</v>
       </c>
       <c r="D16" t="str">
+        <v>Ремонт фар JAGUAR</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Особенности ремонта фар JAGUAR</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Герметизация и «стекло»::Фары JAGUAR из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На JAGUAR светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар JAGUAR чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары JAGUAR собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G16" t="str">
         <v>ремонт фар jaguar</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
-      </c>
-      <c r="F16" t="str">
-        <v>Ремонт и тюнинг фар JAGUAR в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G16" t="str">
-        <v>ремонт фар jaguar, ремонт фар jaguar спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H16" t="str">
         <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
       </c>
       <c r="I16" t="str">
+        <v>Ремонт и тюнинг фар JAGUAR в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J16" t="str">
+        <v>ремонт фар jaguar, ремонт фар jaguar спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
+      </c>
+      <c r="L16" t="str">
         <v>Ремонт и тюнинг фар JAGUAR в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -874,21 +1018,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-jeep_logo.svg.png</v>
       </c>
       <c r="D17" t="str">
+        <v>Ремонт фар JEEP</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Особенности ремонта фар JEEP</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Герметизация и «стекло»::Фары JEEP из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На JEEP светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар JEEP чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары JEEP собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G17" t="str">
         <v>ремонт фар jeep</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
-      </c>
-      <c r="F17" t="str">
-        <v>Ремонт и тюнинг фар JEEP в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G17" t="str">
-        <v>ремонт фар jeep, ремонт фар jeep спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H17" t="str">
         <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
       </c>
       <c r="I17" t="str">
+        <v>Ремонт и тюнинг фар JEEP в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J17" t="str">
+        <v>ремонт фар jeep, ремонт фар jeep спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
+      </c>
+      <c r="L17" t="str">
         <v>Ремонт и тюнинг фар JEEP в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -903,21 +1056,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/kia.webp</v>
       </c>
       <c r="D18" t="str">
+        <v>Ремонт фар KIA</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Особенности ремонта фар KIA</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Герметизация и «стекло»::Фары KIA из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На KIA светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар KIA чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары KIA собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G18" t="str">
         <v>ремонт фар kia</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
-      </c>
-      <c r="F18" t="str">
-        <v>Ремонт и тюнинг фар KIA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G18" t="str">
-        <v>ремонт фар kia, ремонт фар kia спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H18" t="str">
         <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
       </c>
       <c r="I18" t="str">
+        <v>Ремонт и тюнинг фар KIA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J18" t="str">
+        <v>ремонт фар kia, ремонт фар kia спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
+      </c>
+      <c r="L18" t="str">
         <v>Ремонт и тюнинг фар KIA в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -932,21 +1094,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ktm.svg</v>
       </c>
       <c r="D19" t="str">
+        <v>Ремонт фар KTM</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Особенности ремонта фар KTM</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Герметизация и «стекло»::Фары KTM из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На KTM светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар KTM чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары KTM собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G19" t="str">
         <v>ремонт фар ktm</v>
-      </c>
-      <c r="E19" t="str">
-        <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
-      </c>
-      <c r="F19" t="str">
-        <v>Ремонт и тюнинг фар KTM в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G19" t="str">
-        <v>ремонт фар ktm, ремонт фар ktm спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H19" t="str">
         <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
       </c>
       <c r="I19" t="str">
+        <v>Ремонт и тюнинг фар KTM в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J19" t="str">
+        <v>ремонт фар ktm, ремонт фар ktm спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
+      </c>
+      <c r="L19" t="str">
         <v>Ремонт и тюнинг фар KTM в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -961,21 +1132,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/land-rover.svg</v>
       </c>
       <c r="D20" t="str">
+        <v>Ремонт фар Land Rover</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Особенности ремонта фар Land Rover</v>
+      </c>
+      <c r="F20" t="str">
+        <v>LED-секции и ДХО::У Range Rover / Evoque часто выгорают полосы ДХО и модули ближнего. Нужна точечная замена секций и драйверов, а не вся фара целиком.|Герметизация и стёкла::Поликарбонат мутнеет и царапается. Правильный ремонт — снятие старого лака, шлифовка и новый УФ-защитный слой, иначе через сезон фара снова «мутная».|Запотевание и мембраны::Корпуса Land Rover чувствительны к забитым мембранам. Герметизация без дренажа превращает фару в «аквариум» и убивает электронику.|Разбор и линзы::Вскрытие по штатному герметику требует нагрева. Меняем линзы и LED-модули с сохранением геометрии корпуса и герметичности.</v>
+      </c>
+      <c r="G20" t="str">
         <v>ремонт фар land rover</v>
-      </c>
-      <c r="E20" t="str">
-        <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
-      </c>
-      <c r="F20" t="str">
-        <v>Ремонт и тюнинг фар Land Rover в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G20" t="str">
-        <v>ремонт фар land rover, ремонт фар land rover спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H20" t="str">
         <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
       </c>
       <c r="I20" t="str">
+        <v>Ремонт и тюнинг фар Land Rover в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J20" t="str">
+        <v>ремонт фар land rover, ремонт фар land rover спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
+      </c>
+      <c r="L20" t="str">
         <v>Ремонт и тюнинг фар Land Rover в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -990,21 +1170,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/lexus.webp</v>
       </c>
       <c r="D21" t="str">
+        <v>Ремонт фар LEXUS</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Особенности ремонта фар LEXUS</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Герметизация и «стекло»::Фары LEXUS из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На LEXUS светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар LEXUS чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары LEXUS собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G21" t="str">
         <v>ремонт фар lexus</v>
-      </c>
-      <c r="E21" t="str">
-        <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
-      </c>
-      <c r="F21" t="str">
-        <v>Ремонт и тюнинг фар LEXUS в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G21" t="str">
-        <v>ремонт фар lexus, ремонт фар lexus спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H21" t="str">
         <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
       </c>
       <c r="I21" t="str">
+        <v>Ремонт и тюнинг фар LEXUS в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J21" t="str">
+        <v>ремонт фар lexus, ремонт фар lexus спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
+      </c>
+      <c r="L21" t="str">
         <v>Ремонт и тюнинг фар LEXUS в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1019,21 +1208,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/maserati_logo.svg</v>
       </c>
       <c r="D22" t="str">
+        <v>Ремонт фар Maserati</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Особенности ремонта фар Maserati</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Герметизация и «стекло»::Фары Maserati из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На Maserati светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар Maserati чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары Maserati собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G22" t="str">
         <v>ремонт фар maserati</v>
-      </c>
-      <c r="E22" t="str">
-        <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
-      </c>
-      <c r="F22" t="str">
-        <v>Ремонт и тюнинг фар Maserati в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G22" t="str">
-        <v>ремонт фар maserati, ремонт фар maserati спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H22" t="str">
         <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
       </c>
       <c r="I22" t="str">
+        <v>Ремонт и тюнинг фар Maserati в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J22" t="str">
+        <v>ремонт фар maserati, ремонт фар maserati спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
+      </c>
+      <c r="L22" t="str">
         <v>Ремонт и тюнинг фар Maserati в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1048,21 +1246,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/maybach.svg</v>
       </c>
       <c r="D23" t="str">
+        <v>Ремонт фар Maybach</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Особенности ремонта фар Maybach</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Герметизация и «стекло»::Фары Maybach из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На Maybach светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар Maybach чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары Maybach собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G23" t="str">
         <v>ремонт фар maybach</v>
-      </c>
-      <c r="E23" t="str">
-        <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
-      </c>
-      <c r="F23" t="str">
-        <v>Ремонт и тюнинг фар Maybach в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G23" t="str">
-        <v>ремонт фар maybach, ремонт фар maybach спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H23" t="str">
         <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
       </c>
       <c r="I23" t="str">
+        <v>Ремонт и тюнинг фар Maybach в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J23" t="str">
+        <v>ремонт фар maybach, ремонт фар maybach спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
+      </c>
+      <c r="L23" t="str">
         <v>Ремонт и тюнинг фар Maybach в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1077,21 +1284,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mazda.svg</v>
       </c>
       <c r="D24" t="str">
+        <v>Ремонт фар MAZDA</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Особенности ремонта фар MAZDA</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Герметизация и «стекло»::Фары MAZDA из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На MAZDA светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар MAZDA чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары MAZDA собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G24" t="str">
         <v>ремонт фар mazda</v>
-      </c>
-      <c r="E24" t="str">
-        <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
-      </c>
-      <c r="F24" t="str">
-        <v>Ремонт и тюнинг фар MAZDA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G24" t="str">
-        <v>ремонт фар mazda, ремонт фар mazda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H24" t="str">
         <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
       </c>
       <c r="I24" t="str">
+        <v>Ремонт и тюнинг фар MAZDA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J24" t="str">
+        <v>ремонт фар mazda, ремонт фар mazda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
+      </c>
+      <c r="L24" t="str">
         <v>Ремонт и тюнинг фар MAZDA в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1106,21 +1322,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mercedes.webp</v>
       </c>
       <c r="D25" t="str">
+        <v>Ремонт фар MERCEDES</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Особенности ремонта фар MERCEDES</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Multibeam и ILS::На Mercedes (W213, W222, X253) сложные Multibeam/ILS-блоки. Проблемы часто в платах управления и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Герметизация и «стекло»::Стёкла мутнеют и царапаются. Грубая полировка убивает заводской УФ-лак. Восстанавливаем прозрачность со снятием старого покрытия и нанесением нового защитного слоя.|Разгерметизация и дренаж::Запотевание обычно связано с мембранами и вентиляцией корпуса. Просто «промазать шов» без замены дренажа усугубляет конденсат и повреждает электронику.|Неразборный корпус::Фары на современном герметике требуют точного нагрева при разборе. Любительское вскрытие даёт трещины. Линзы и LED-модули меняем с ювелирной пайкой и проверкой на стенде.</v>
+      </c>
+      <c r="G25" t="str">
         <v>ремонт фар mercedes</v>
-      </c>
-      <c r="E25" t="str">
-        <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
-      </c>
-      <c r="F25" t="str">
-        <v>Ремонт и тюнинг фар MERCEDES в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G25" t="str">
-        <v>ремонт фар mercedes, ремонт фар mercedes спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H25" t="str">
         <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
       </c>
       <c r="I25" t="str">
+        <v>Ремонт и тюнинг фар MERCEDES в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J25" t="str">
+        <v>ремонт фар mercedes, ремонт фар mercedes спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
+      </c>
+      <c r="L25" t="str">
         <v>Ремонт и тюнинг фар MERCEDES в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1135,21 +1360,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mini-logo.png</v>
       </c>
       <c r="D26" t="str">
+        <v>Ремонт фар MINI</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Особенности ремонта фар MINI</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Герметизация и «стекло»::Фары MINI из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На MINI светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар MINI чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары MINI собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G26" t="str">
         <v>ремонт фар mini</v>
-      </c>
-      <c r="E26" t="str">
-        <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
-      </c>
-      <c r="F26" t="str">
-        <v>Ремонт и тюнинг фар MINI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G26" t="str">
-        <v>ремонт фар mini, ремонт фар mini спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H26" t="str">
         <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
       </c>
       <c r="I26" t="str">
+        <v>Ремонт и тюнинг фар MINI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J26" t="str">
+        <v>ремонт фар mini, ремонт фар mini спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
+      </c>
+      <c r="L26" t="str">
         <v>Ремонт и тюнинг фар MINI в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1164,21 +1398,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/mitsubishi.svg</v>
       </c>
       <c r="D27" t="str">
+        <v>Ремонт фар MITSUBISHI</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Особенности ремонта фар MITSUBISHI</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Герметизация и «стекло»::Фары MITSUBISHI из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На MITSUBISHI светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар MITSUBISHI чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары MITSUBISHI собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G27" t="str">
         <v>ремонт фар mitsubishi</v>
-      </c>
-      <c r="E27" t="str">
-        <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
-      </c>
-      <c r="F27" t="str">
-        <v>Ремонт и тюнинг фар MITSUBISHI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G27" t="str">
-        <v>ремонт фар mitsubishi, ремонт фар mitsubishi спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H27" t="str">
         <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
       </c>
       <c r="I27" t="str">
+        <v>Ремонт и тюнинг фар MITSUBISHI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J27" t="str">
+        <v>ремонт фар mitsubishi, ремонт фар mitsubishi спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
+      </c>
+      <c r="L27" t="str">
         <v>Ремонт и тюнинг фар MITSUBISHI в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1193,21 +1436,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-nissan_logo.svg.png</v>
       </c>
       <c r="D28" t="str">
+        <v>Ремонт фар NISSAN</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Особенности ремонта фар NISSAN</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Герметизация и «стекло»::Фары NISSAN из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На NISSAN светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар NISSAN чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары NISSAN собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G28" t="str">
         <v>ремонт фар nissan</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
-      </c>
-      <c r="F28" t="str">
-        <v>Ремонт и тюнинг фар NISSAN в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G28" t="str">
-        <v>ремонт фар nissan, ремонт фар nissan спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H28" t="str">
         <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
       </c>
       <c r="I28" t="str">
+        <v>Ремонт и тюнинг фар NISSAN в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J28" t="str">
+        <v>ремонт фар nissan, ремонт фар nissan спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
+      </c>
+      <c r="L28" t="str">
         <v>Ремонт и тюнинг фар NISSAN в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1222,21 +1474,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/opel.svg</v>
       </c>
       <c r="D29" t="str">
+        <v>Ремонт фар OPEL</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Особенности ремонта фар OPEL</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Герметизация и «стекло»::Фары OPEL из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На OPEL светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар OPEL чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары OPEL собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G29" t="str">
         <v>ремонт фар opel</v>
-      </c>
-      <c r="E29" t="str">
-        <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
-      </c>
-      <c r="F29" t="str">
-        <v>Ремонт и тюнинг фар OPEL в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G29" t="str">
-        <v>ремонт фар opel, ремонт фар opel спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H29" t="str">
         <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
       </c>
       <c r="I29" t="str">
+        <v>Ремонт и тюнинг фар OPEL в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J29" t="str">
+        <v>ремонт фар opel, ремонт фар opel спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
+      </c>
+      <c r="L29" t="str">
         <v>Ремонт и тюнинг фар OPEL в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1251,21 +1512,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/peugeot.svg</v>
       </c>
       <c r="D30" t="str">
+        <v>Ремонт фар PEUGEOT</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Особенности ремонта фар PEUGEOT</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Герметизация и «стекло»::Фары PEUGEOT из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На PEUGEOT светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар PEUGEOT чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары PEUGEOT собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G30" t="str">
         <v>ремонт фар peugeot</v>
-      </c>
-      <c r="E30" t="str">
-        <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
-      </c>
-      <c r="F30" t="str">
-        <v>Ремонт и тюнинг фар PEUGEOT в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G30" t="str">
-        <v>ремонт фар peugeot, ремонт фар peugeot спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H30" t="str">
         <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
       </c>
       <c r="I30" t="str">
+        <v>Ремонт и тюнинг фар PEUGEOT в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J30" t="str">
+        <v>ремонт фар peugeot, ремонт фар peugeot спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
+      </c>
+      <c r="L30" t="str">
         <v>Ремонт и тюнинг фар PEUGEOT в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1280,21 +1550,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/porsche-logo.png</v>
       </c>
       <c r="D31" t="str">
+        <v>Ремонт фар PORSCHE</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Особенности ремонта фар PORSCHE</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Матричные и PDLS-системы::На Porsche фары тесно связаны с блоками PDLS/матричного света. Ошибки часто в драйверах и шине, а не в самом диоде. Нужна диагностика и точечный ремонт плат.|Герметизация и «стекло»::Поликарбонат мутнеет быстро на трассе. Грубая полировка снимает УФ-лак навсегда. Делаем полное восстановление покрытия, а не «глянец на неделю».|Разгерметизация и дренаж::Запотевание почти всегда связано с мембранами. Без их замены любая герметизация шва даёт обратный эффект.|Неразборный корпус и линзы::Корпуса на жёстком герметике. Вскрытие только с контролем температуры. Замена линз — аккуратная работа с сохранением штатной оптики пучка.</v>
+      </c>
+      <c r="G31" t="str">
         <v>ремонт фар porsche</v>
-      </c>
-      <c r="E31" t="str">
-        <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
-      </c>
-      <c r="F31" t="str">
-        <v>Ремонт и тюнинг фар PORSCHE в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G31" t="str">
-        <v>ремонт фар porsche, ремонт фар porsche спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H31" t="str">
         <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
       </c>
       <c r="I31" t="str">
+        <v>Ремонт и тюнинг фар PORSCHE в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J31" t="str">
+        <v>ремонт фар porsche, ремонт фар porsche спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
+      </c>
+      <c r="L31" t="str">
         <v>Ремонт и тюнинг фар PORSCHE в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1309,21 +1588,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/renault-logo.png</v>
       </c>
       <c r="D32" t="str">
+        <v>Ремонт фар RENAULT</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Особенности ремонта фар RENAULT</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Герметизация и «стекло»::Фары RENAULT из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На RENAULT светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар RENAULT чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары RENAULT собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G32" t="str">
         <v>ремонт фар renault</v>
-      </c>
-      <c r="E32" t="str">
-        <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
-      </c>
-      <c r="F32" t="str">
-        <v>Ремонт и тюнинг фар RENAULT в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G32" t="str">
-        <v>ремонт фар renault, ремонт фар renault спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H32" t="str">
         <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
       </c>
       <c r="I32" t="str">
+        <v>Ремонт и тюнинг фар RENAULT в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J32" t="str">
+        <v>ремонт фар renault, ремонт фар renault спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
+      </c>
+      <c r="L32" t="str">
         <v>Ремонт и тюнинг фар RENAULT в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1338,21 +1626,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/500px-rolls-royce_motor_cars_logo.svg.png</v>
       </c>
       <c r="D33" t="str">
+        <v>Ремонт фар Rolls-Royce</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Особенности ремонта фар Rolls-Royce</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Герметизация и «стекло»::Фары Rolls-Royce из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На Rolls-Royce светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар Rolls-Royce чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары Rolls-Royce собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G33" t="str">
         <v>ремонт фар rolls-royce</v>
-      </c>
-      <c r="E33" t="str">
-        <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
-      </c>
-      <c r="F33" t="str">
-        <v>Ремонт и тюнинг фар Rolls-Royce в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G33" t="str">
-        <v>ремонт фар rolls-royce, ремонт фар rolls-royce спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H33" t="str">
         <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
       </c>
       <c r="I33" t="str">
+        <v>Ремонт и тюнинг фар Rolls-Royce в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J33" t="str">
+        <v>ремонт фар rolls-royce, ремонт фар rolls-royce спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
+      </c>
+      <c r="L33" t="str">
         <v>Ремонт и тюнинг фар Rolls-Royce в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1367,21 +1664,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/saab.svg</v>
       </c>
       <c r="D34" t="str">
+        <v>Ремонт фар SAAB</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Особенности ремонта фар SAAB</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Герметизация и «стекло»::Фары SAAB из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На SAAB светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар SAAB чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары SAAB собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G34" t="str">
         <v>ремонт фар saab</v>
-      </c>
-      <c r="E34" t="str">
-        <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
-      </c>
-      <c r="F34" t="str">
-        <v>Ремонт и тюнинг фар SAAB в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G34" t="str">
-        <v>ремонт фар saab, ремонт фар saab спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H34" t="str">
         <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
       </c>
       <c r="I34" t="str">
+        <v>Ремонт и тюнинг фар SAAB в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J34" t="str">
+        <v>ремонт фар saab, ремонт фар saab спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
+      </c>
+      <c r="L34" t="str">
         <v>Ремонт и тюнинг фар SAAB в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1396,21 +1702,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/skoda.svg</v>
       </c>
       <c r="D35" t="str">
+        <v>Ремонт фар Skoda</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Особенности ремонта фар Skoda</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Герметизация и «стекло»::Фары Skoda из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На Skoda светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар Skoda чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары Skoda собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G35" t="str">
         <v>ремонт фар skoda</v>
-      </c>
-      <c r="E35" t="str">
-        <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
-      </c>
-      <c r="F35" t="str">
-        <v>Ремонт и тюнинг фар Skoda в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G35" t="str">
-        <v>ремонт фар skoda, ремонт фар skoda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H35" t="str">
         <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
       </c>
       <c r="I35" t="str">
+        <v>Ремонт и тюнинг фар Skoda в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J35" t="str">
+        <v>ремонт фар skoda, ремонт фар skoda спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
+      </c>
+      <c r="L35" t="str">
         <v>Ремонт и тюнинг фар Skoda в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1425,21 +1740,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/ssangyong-logo.png</v>
       </c>
       <c r="D36" t="str">
+        <v>Ремонт фар SsangYong</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Особенности ремонта фар SsangYong</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Герметизация и «стекло»::Фары SsangYong из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На SsangYong светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар SsangYong чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары SsangYong собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G36" t="str">
         <v>ремонт фар ssangyong</v>
-      </c>
-      <c r="E36" t="str">
-        <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
-      </c>
-      <c r="F36" t="str">
-        <v>Ремонт и тюнинг фар SsangYong в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G36" t="str">
-        <v>ремонт фар ssangyong, ремонт фар ssangyong спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H36" t="str">
         <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
       </c>
       <c r="I36" t="str">
+        <v>Ремонт и тюнинг фар SsangYong в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J36" t="str">
+        <v>ремонт фар ssangyong, ремонт фар ssangyong спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
+      </c>
+      <c r="L36" t="str">
         <v>Ремонт и тюнинг фар SsangYong в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1454,21 +1778,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/subaru-logo.png</v>
       </c>
       <c r="D37" t="str">
+        <v>Ремонт фар SUBARU</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Особенности ремонта фар SUBARU</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Герметизация и «стекло»::Фары SUBARU из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На SUBARU светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар SUBARU чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары SUBARU собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G37" t="str">
         <v>ремонт фар subaru</v>
-      </c>
-      <c r="E37" t="str">
-        <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
-      </c>
-      <c r="F37" t="str">
-        <v>Ремонт и тюнинг фар SUBARU в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G37" t="str">
-        <v>ремонт фар subaru, ремонт фар subaru спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H37" t="str">
         <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
       </c>
       <c r="I37" t="str">
+        <v>Ремонт и тюнинг фар SUBARU в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J37" t="str">
+        <v>ремонт фар subaru, ремонт фар subaru спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
+      </c>
+      <c r="L37" t="str">
         <v>Ремонт и тюнинг фар SUBARU в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1483,21 +1816,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/suzuki.svg</v>
       </c>
       <c r="D38" t="str">
+        <v>Ремонт фар SUZUKI</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Особенности ремонта фар SUZUKI</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Герметизация и «стекло»::Фары SUZUKI из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На SUZUKI светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар SUZUKI чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары SUZUKI собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G38" t="str">
         <v>ремонт фар suzuki</v>
-      </c>
-      <c r="E38" t="str">
-        <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
-      </c>
-      <c r="F38" t="str">
-        <v>Ремонт и тюнинг фар SUZUKI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G38" t="str">
-        <v>ремонт фар suzuki, ремонт фар suzuki спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H38" t="str">
         <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
       </c>
       <c r="I38" t="str">
+        <v>Ремонт и тюнинг фар SUZUKI в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J38" t="str">
+        <v>ремонт фар suzuki, ремонт фар suzuki спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
+      </c>
+      <c r="L38" t="str">
         <v>Ремонт и тюнинг фар SUZUKI в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1512,21 +1854,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/toyota.webp</v>
       </c>
       <c r="D39" t="str">
+        <v>Ремонт фар TOYOTA</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Особенности ремонта фар TOYOTA</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Герметизация и «стекло»::Фары TOYOTA из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На TOYOTA светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар TOYOTA чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары TOYOTA собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G39" t="str">
         <v>ремонт фар toyota</v>
-      </c>
-      <c r="E39" t="str">
-        <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
-      </c>
-      <c r="F39" t="str">
-        <v>Ремонт и тюнинг фар TOYOTA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G39" t="str">
-        <v>ремонт фар toyota, ремонт фар toyota спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H39" t="str">
         <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
       </c>
       <c r="I39" t="str">
+        <v>Ремонт и тюнинг фар TOYOTA в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J39" t="str">
+        <v>ремонт фар toyota, ремонт фар toyota спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
+      </c>
+      <c r="L39" t="str">
         <v>Ремонт и тюнинг фар TOYOTA в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1541,21 +1892,30 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/volkswagen.webp</v>
       </c>
       <c r="D40" t="str">
+        <v>Ремонт фар Volkswagen</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Особенности ремонта фар Volkswagen</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Герметизация и «стекло»::Фары Volkswagen из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На Volkswagen светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар Volkswagen чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары Volkswagen собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G40" t="str">
         <v>ремонт фар volkswagen</v>
-      </c>
-      <c r="E40" t="str">
-        <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
-      </c>
-      <c r="F40" t="str">
-        <v>Ремонт и тюнинг фар Volkswagen в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G40" t="str">
-        <v>ремонт фар volkswagen, ремонт фар volkswagen спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H40" t="str">
         <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
       </c>
       <c r="I40" t="str">
+        <v>Ремонт и тюнинг фар Volkswagen в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J40" t="str">
+        <v>ремонт фар volkswagen, ремонт фар volkswagen спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
+      </c>
+      <c r="L40" t="str">
         <v>Ремонт и тюнинг фар Volkswagen в СПб | КБ АВТО</v>
       </c>
     </row>
@@ -1570,27 +1930,36 @@
         <v>http://ksenonspby.temp.swtest.ru/wp-content/uploads/2026/07/volvo.svg</v>
       </c>
       <c r="D41" t="str">
+        <v>Ремонт фар VOLVO</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Особенности ремонта фар VOLVO</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Герметизация и «стекло»::Фары VOLVO из поликарбоната мутнеют и царапаются. Заводской лак твёрдый, но тонкий: грубая полировка стирает УФ-защиту. Правильный ремонт — снятие старого лака, шлифовка и новый двухкомпонентный защитный слой.|Электроника и датчики::На VOLVO светодиодные и адаптивные фары связаны с блоками управления. Часто проблема в драйверах, шлейфах и датчиках, а не в «сгоревшей лампе». Нужны диагностика и микроэлектронный ремонт.|Разгерметизация и дренаж::Запотевание фар VOLVO чаще вызвано забитыми мембранами и вентиляцией, а не только трещиной. Герметизация шва без замены дренажа превращает корпус в «аквариум».|Неразборный корпус и линзы::Современные фары VOLVO собраны на жёстком герметике. Вскрытие требует точного нагрева. Замена линз и LED-модулей — аккуратная пайка с сохранением герметичности и геометрии пучка.</v>
+      </c>
+      <c r="G41" t="str">
         <v>ремонт фар volvo</v>
-      </c>
-      <c r="E41" t="str">
-        <v>Ремонт и тюнинг фар VOLVO в СПб | КБ АВТО</v>
-      </c>
-      <c r="F41" t="str">
-        <v>Ремонт и тюнинг фар VOLVO в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
-      </c>
-      <c r="G41" t="str">
-        <v>ремонт фар volvo, ремонт фар volvo спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
       <c r="H41" t="str">
         <v>Ремонт и тюнинг фар VOLVO в СПб | КБ АВТО</v>
       </c>
       <c r="I41" t="str">
+        <v>Ремонт и тюнинг фар VOLVO в Санкт-Петербурге — восстановление оптики, установка линз, устранение запотевания. КБ АВТО, Санкт-Петербург.</v>
+      </c>
+      <c r="J41" t="str">
+        <v>ремонт фар volvo, ремонт фар volvo спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
+      </c>
+      <c r="K41" t="str">
+        <v>Ремонт и тюнинг фар VOLVO в СПб | КБ АВТО</v>
+      </c>
+      <c r="L41" t="str">
         <v>Ремонт и тюнинг фар VOLVO в СПб | КБ АВТО</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>